<commit_message>
feat: add BA bulk template files with signature URL fields
</commit_message>
<xml_diff>
--- a/resources/templates/payslip-bulk-template.xlsx
+++ b/resources/templates/payslip-bulk-template.xlsx
@@ -401,108 +401,108 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
+        <v>employeeID</v>
+      </c>
+      <c r="B1" t="str">
+        <v>employeeName</v>
+      </c>
+      <c r="C1" t="str">
+        <v>position</v>
+      </c>
+      <c r="D1" t="str">
+        <v>departement</v>
+      </c>
+      <c r="E1" t="str">
+        <v>ptkp</v>
+      </c>
+      <c r="F1" t="str">
+        <v>periode</v>
+      </c>
+      <c r="G1" t="str">
+        <v>joinDate</v>
+      </c>
+      <c r="H1" t="str">
+        <v>targetHK</v>
+      </c>
+      <c r="I1" t="str">
+        <v>attendance</v>
+      </c>
+      <c r="J1" t="str">
+        <v>Gaji Pokok</v>
+      </c>
+      <c r="K1" t="str">
+        <v>Tunjangan makan</v>
+      </c>
+      <c r="L1" t="str">
+        <v>Tunjangan Transport</v>
+      </c>
+      <c r="M1" t="str">
+        <v>Tunjangan Komunikasi</v>
+      </c>
+      <c r="N1" t="str">
+        <v>Tunjangan Jabatan</v>
+      </c>
+      <c r="O1" t="str">
+        <v>BPJS Ketenagakerjaan</v>
+      </c>
+      <c r="P1" t="str">
+        <v>PPH 21</v>
+      </c>
+      <c r="Q1" t="str">
         <v>email</v>
-      </c>
-      <c r="B1" t="str">
-        <v>employeeID</v>
-      </c>
-      <c r="C1" t="str">
-        <v>employeeName</v>
-      </c>
-      <c r="D1" t="str">
-        <v>position</v>
-      </c>
-      <c r="E1" t="str">
-        <v>departement</v>
-      </c>
-      <c r="F1" t="str">
-        <v>ptkp</v>
-      </c>
-      <c r="G1" t="str">
-        <v>periode</v>
-      </c>
-      <c r="H1" t="str">
-        <v>joinDate</v>
-      </c>
-      <c r="I1" t="str">
-        <v>targetHK</v>
-      </c>
-      <c r="J1" t="str">
-        <v>attendance</v>
-      </c>
-      <c r="K1" t="str">
-        <v>Gaji Pokok</v>
-      </c>
-      <c r="L1" t="str">
-        <v>Tunjangan makan</v>
-      </c>
-      <c r="M1" t="str">
-        <v>Tunjangan Transport</v>
-      </c>
-      <c r="N1" t="str">
-        <v>Tunjangan Komunikasi</v>
-      </c>
-      <c r="O1" t="str">
-        <v>Tunjangan Jabatan</v>
-      </c>
-      <c r="P1" t="str">
-        <v>BPJS Ketenagakerjaan</v>
-      </c>
-      <c r="Q1" t="str">
-        <v>PPH 21</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>karyawan@example.com</v>
+        <v>EMP-001</v>
       </c>
       <c r="B2" t="str">
-        <v>EMP-001</v>
+        <v>Budi Santoso</v>
       </c>
       <c r="C2" t="str">
-        <v>Budi Santoso</v>
+        <v>Software Engineer</v>
       </c>
       <c r="D2" t="str">
-        <v>Software Engineer</v>
+        <v>IT</v>
       </c>
       <c r="E2" t="str">
-        <v>IT</v>
+        <v>TK0</v>
       </c>
       <c r="F2" t="str">
-        <v>TK0</v>
+        <v>Maret 2026</v>
       </c>
       <c r="G2" t="str">
-        <v>Maret 2026</v>
+        <v>2024-08-01</v>
       </c>
       <c r="H2" t="str">
-        <v>2024-08-01</v>
+        <v>22</v>
       </c>
       <c r="I2" t="str">
-        <v>22</v>
-      </c>
-      <c r="J2" t="str">
         <v>21/22</v>
       </c>
+      <c r="J2">
+        <v>12000000</v>
+      </c>
       <c r="K2">
-        <v>12000000</v>
+        <v>800000</v>
       </c>
       <c r="L2">
+        <v>1000000</v>
+      </c>
+      <c r="M2">
         <v>800000</v>
-      </c>
-      <c r="M2">
-        <v>1000000</v>
       </c>
       <c r="N2">
         <v>800000</v>
       </c>
       <c r="O2">
-        <v>800000</v>
+        <v>300000</v>
       </c>
       <c r="P2">
-        <v>300000</v>
-      </c>
-      <c r="Q2">
         <v>250000</v>
+      </c>
+      <c r="Q2" t="str">
+        <v>user@example.com</v>
       </c>
     </row>
   </sheetData>

</xml_diff>